<commit_message>
Electrical architecture, wiring blueprint, wheeled gear proposal and NWA sponsorship
- docs/research/electrical-architecture.md + inventory/electrical/*.json:
  power and signal trees, FC output/UART map (ArduPilot QuadPlane), power
  budget, wire gauges, connectors, breakdown joints J1-J3, test plan,
  wheeled landing gear geometry (pusher clearance 36 -> 84 mm EST)
- Inventory-Overview.html: 3D model now shows avionics, ESCs, servos, wire
  runs and proposed wheels; new Electrical and Wiring & tests sections
  (blueprint DBF-ELE-001, wire schedule, harness by joint); gear proposal;
  NWA founders' verbal sponsorship offer with a message to send
- inventory: NWA status, proposed lines G-01..G-04 kept out of committed
  spend; sheet seed adds proposed-spend rows
- README: section 3, layout, open items

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BoGkgR3KP795byqnkkcvJ5
</commit_message>
<xml_diff>
--- a/inventory/DBF-Inventory.xlsx
+++ b/inventory/DBF-Inventory.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inventory'!$A$1:$W$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inventory'!$A$1:$W$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1137,7 +1137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W64"/>
+  <dimension ref="A1:W68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="K63" s="16" t="inlineStr">
         <is>
-          <t>Proposed: confirm with NWA</t>
+          <t>Proposed: NWA sponsor offer (verbal)</t>
         </is>
       </c>
       <c r="L63" s="14" t="inlineStr">
@@ -6225,12 +6225,12 @@
       <c r="U63" s="16" t="n"/>
       <c r="V63" s="15" t="inlineStr">
         <is>
-          <t>docs/research/nautical-wings-props.md</t>
+          <t>docs/research/nautical-wings-props.md; sponsorship: team-reported (founders, in person, Oct 2026)</t>
         </is>
       </c>
       <c r="W63" s="20" t="inlineStr">
         <is>
-          <t>Replaces JeeFly 1755 x 6 if confirmed. Fit to X4110S bolt-on adapter (4 mm shaft); hover point 15.2 N per rotor</t>
+          <t>NWA founders offered to sponsor the team (met in person; team-reported, Oct 2026). Sponsorship rules not yet confirmed in writing. Replaces JeeFly 1755 x 6 if confirmed. Fit to X4110S bolt-on adapter (4 mm shaft); hover point 15.2 N per rotor</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6280,7 @@
       </c>
       <c r="K64" s="16" t="inlineStr">
         <is>
-          <t>Proposed: confirm with NWA</t>
+          <t>Proposed: NWA sponsor offer (verbal)</t>
         </is>
       </c>
       <c r="L64" s="14" t="inlineStr">
@@ -6312,17 +6312,345 @@
       <c r="U64" s="16" t="n"/>
       <c r="V64" s="15" t="inlineStr">
         <is>
-          <t>docs/research/nautical-wings-props.md</t>
+          <t>docs/research/nautical-wings-props.md; sponsorship: team-reported (founders, in person, Oct 2026)</t>
         </is>
       </c>
       <c r="W64" s="20" t="inlineStr">
         <is>
-          <t>Replaces APC 14x8.5EP x 3 if confirmed; keep one APC as thrust-stand baseline (team call)</t>
+          <t>NWA founders offered to sponsor the team (met in person; team-reported, Oct 2026). Sponsorship rules not yet confirmed in writing. Replaces APC 14x8.5EP x 3 if confirmed; keep one APC as thrust-stand baseline (team call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>G-01</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>Du-Bro Super Lite 3.00 in wheel pair (SKU 300SL, 16.8 g/wheel, 5/32 in axle)</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>Landing gear</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>Landing_Leg</t>
+        </is>
+      </c>
+      <c r="G65" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="14">
+        <f>MAX(0,G65-I65-N(H65))</f>
+        <v/>
+      </c>
+      <c r="K65" s="16" t="inlineStr">
+        <is>
+          <t>Proposed: wheeled gear</t>
+        </is>
+      </c>
+      <c r="L65" s="14" t="inlineStr">
+        <is>
+          <t>Gator RC</t>
+        </is>
+      </c>
+      <c r="M65" s="17" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="N65" s="17">
+        <f>G65*M65</f>
+        <v/>
+      </c>
+      <c r="O65" s="18" t="n"/>
+      <c r="P65" s="14" t="n"/>
+      <c r="Q65" s="15" t="n"/>
+      <c r="R65" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S65" s="19" t="n"/>
+      <c r="T65" s="19" t="n"/>
+      <c r="U65" s="16" t="n"/>
+      <c r="V65" s="15" t="inlineStr">
+        <is>
+          <t>inventory/electrical/proposed_lines.json: https://www.gator-rc.com/products/dubro-super-lite-wheels (checked 2026-10-19)</t>
+        </is>
+      </c>
+      <c r="W65" s="20" t="inlineStr">
+        <is>
+          <t>Landing gear on the four existing legs (2 pairs = 4 wheels); raises ground plane 0.048 m EST (wheel radius 0.0381 m + 10 mm axle offset EST), pusher disc clearance 36 to 84 mm. Gator RC page read 2026-10-19: $6.75 per pair, 'Only 1 left' for the product, so one pair must come from another vendor; re-quote before ordering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>G-02</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>Du-Bro axle shaft 2-pack, 5/32 in x 2 in (DUB248), with 2 nylon-insert nuts</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>Landing gear</t>
+        </is>
+      </c>
+      <c r="E66" s="14" t="inlineStr">
+        <is>
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
+          <t>Landing_Leg</t>
+        </is>
+      </c>
+      <c r="G66" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H66" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="14">
+        <f>MAX(0,G66-I66-N(H66))</f>
+        <v/>
+      </c>
+      <c r="K66" s="16" t="inlineStr">
+        <is>
+          <t>Proposed: wheeled gear</t>
+        </is>
+      </c>
+      <c r="L66" s="14" t="inlineStr">
+        <is>
+          <t>Gator RC</t>
+        </is>
+      </c>
+      <c r="M66" s="17" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="N66" s="17">
+        <f>G66*M66</f>
+        <v/>
+      </c>
+      <c r="O66" s="18" t="n"/>
+      <c r="P66" s="14" t="n"/>
+      <c r="Q66" s="15" t="n"/>
+      <c r="R66" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S66" s="19" t="n"/>
+      <c r="T66" s="19" t="n"/>
+      <c r="U66" s="16" t="n"/>
+      <c r="V66" s="15" t="inlineStr">
+        <is>
+          <t>inventory/electrical/proposed_lines.json: https://www.gator-rc.com/products/du-bro-rc-airplane-axle-shafts-2-pack (checked 2026-10-19)</t>
+        </is>
+      </c>
+      <c r="W66" s="20" t="inlineStr">
+        <is>
+          <t>Four axles for four wheels; thread size not published (—), fit-check against leg tip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>G-03</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>Du-Bro 5/32 in wheel collars 4-pack (DUB140)</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>Landing gear</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="F67" s="14" t="inlineStr">
+        <is>
+          <t>Landing_Leg</t>
+        </is>
+      </c>
+      <c r="G67" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H67" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="14">
+        <f>MAX(0,G67-I67-N(H67))</f>
+        <v/>
+      </c>
+      <c r="K67" s="16" t="inlineStr">
+        <is>
+          <t>Proposed: wheeled gear</t>
+        </is>
+      </c>
+      <c r="L67" s="14" t="inlineStr">
+        <is>
+          <t>Gator RC</t>
+        </is>
+      </c>
+      <c r="M67" s="17" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="N67" s="17">
+        <f>G67*M67</f>
+        <v/>
+      </c>
+      <c r="O67" s="18" t="n"/>
+      <c r="P67" s="14" t="n"/>
+      <c r="Q67" s="15" t="n"/>
+      <c r="R67" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S67" s="19" t="n"/>
+      <c r="T67" s="19" t="n"/>
+      <c r="U67" s="16" t="n"/>
+      <c r="V67" s="15" t="inlineStr">
+        <is>
+          <t>inventory/electrical/proposed_lines.json: https://www.gator-rc.com/products/du-bro-wheel-shaft-collars-4-pack (checked 2026-10-19)</t>
+        </is>
+      </c>
+      <c r="W67" s="20" t="inlineStr">
+        <is>
+          <t>Wheel retention; 8 collars, 4 needed, 4 spare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>G-04</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>Panasonic 470 uF 35 V low-ESR capacitor</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="F68" s="14" t="n"/>
+      <c r="G68" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H68" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="14">
+        <f>MAX(0,G68-I68-N(H68))</f>
+        <v/>
+      </c>
+      <c r="K68" s="16" t="inlineStr">
+        <is>
+          <t>Proposed: electrical</t>
+        </is>
+      </c>
+      <c r="L68" s="14" t="inlineStr">
+        <is>
+          <t>Race Day Quads</t>
+        </is>
+      </c>
+      <c r="M68" s="17" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="N68" s="17">
+        <f>G68*M68</f>
+        <v/>
+      </c>
+      <c r="O68" s="18" t="n"/>
+      <c r="P68" s="14" t="n"/>
+      <c r="Q68" s="15" t="n"/>
+      <c r="R68" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S68" s="19" t="n"/>
+      <c r="T68" s="19" t="n"/>
+      <c r="U68" s="16" t="n"/>
+      <c r="V68" s="15" t="inlineStr">
+        <is>
+          <t>inventory/electrical/proposed_lines.json: https://www.racedayquads.com/products/panasonic-470uf-low-esr-capacitor (checked 2026-10-19)</t>
+        </is>
+      </c>
+      <c r="W68" s="20" t="inlineStr">
+        <is>
+          <t>FC battery-side cap (vendor guide) plus one per lift ESC and pusher ESC; stock, size, lead length not on page (—). Voltage 35 V from title only.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W64"/>
+  <autoFilter ref="A1:W68"/>
   <conditionalFormatting sqref="K2:K500">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LEFT($K2,12)="Inspected OK"</formula>
@@ -6652,7 +6980,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Inventory!A1:W64</t>
+          <t>Inventory!A1:W68</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">

</xml_diff>